<commit_message>
Xu ly 3.0: sua nhap ma 6.2, buoc 3, tu tai lai tab; dong goi v1.0.0
Nhap tung ma bang SearchInventory_V2(true), chon buoc chay, doc dung bang 3.2,
tich chon danh sach BD13, khong bam Huy popup in, tai lai tab giua cac buoc.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/extension/assets/mau-import-xuly-30.xlsx
+++ b/extension/assets/mau-import-xuly-30.xlsx
@@ -397,26 +397,35 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:B3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>MA_BG</v>
       </c>
+      <c r="B1" t="str">
+        <v>KET_QUA</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>EL533085492VN</v>
       </c>
+      <c r="B2" t="str">
+        <v>Thành công</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
         <v>EL533240444VN</v>
       </c>
+      <c r="B3" t="str">
+        <v>Thành công</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>